<commit_message>
Add Fund Manager Edition (P3) in English and French
- Fund parameters with generic support profiles, switchable eligibility criteria,
  scoring weights, delivery-by-risk table and concentration limits
- Pipeline of up to 25 projects; eligibility tests with rejection reasons; eight
  normalised scores including additionality against the Developer Edition viability gap
- Non-circular sequential allocation by rank with envelope and country limits
- Tranche-based RBF and grant disbursements, fund cash position, MRV tracker,
  portfolio dashboard and 12 integrity checks
- French dictionary entries, user guides and Etsy/Gumroad listings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BXecWCCHxS2NDKTkshp3of
</commit_message>
<xml_diff>
--- a/product/01-entry-calculator/Calculateur_Faisabilite_MiniReseau_v1_FR.xlsx
+++ b/product/01-entry-calculator/Calculateur_Faisabilite_MiniReseau_v1_FR.xlsx
@@ -2124,8 +2124,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13441805"/>
-        <c:axId val="79404167"/>
+        <c:axId val="23251896"/>
+        <c:axId val="63682204"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2330,11 +2330,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="13441805"/>
-        <c:axId val="79404167"/>
+        <c:axId val="23251896"/>
+        <c:axId val="63682204"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="13441805"/>
+        <c:axId val="23251896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2366,7 +2366,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79404167"/>
+        <c:crossAx val="63682204"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2374,7 +2374,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79404167"/>
+        <c:axId val="63682204"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2450,7 +2450,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13441805"/>
+        <c:crossAx val="23251896"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2921,11 +2921,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="75889040"/>
-        <c:axId val="14482574"/>
+        <c:axId val="4491170"/>
+        <c:axId val="78945054"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75889040"/>
+        <c:axId val="4491170"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2957,7 +2957,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14482574"/>
+        <c:crossAx val="78945054"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2965,7 +2965,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14482574"/>
+        <c:axId val="78945054"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3007,7 +3007,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75889040"/>
+        <c:crossAx val="4491170"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>